<commit_message>
add quantity and make name required
</commit_message>
<xml_diff>
--- a/project/excel/oct_schema.xlsx
+++ b/project/excel/oct_schema.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -422,6 +422,11 @@
           <t>name</t>
         </is>
       </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>quantity</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>